<commit_message>
Rank High side J/K optimization algorithm on a frequency sweep of 25khz spacing from 100khz to 800khz and extracted top 5 mosfets in each bracket
</commit_message>
<xml_diff>
--- a/Mosfet_extraction_pipeline/mosfet_urls.xlsx
+++ b/Mosfet_extraction_pipeline/mosfet_urls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Sync_Buck_convertor\Mosfet_extraction_pipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD33CB36-F88A-4A63-AA44-1F6CC55D3051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14D9E871-3EEA-4943-BABC-0A6C43CA941D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7055,7 +7055,7 @@
     <col min="7" max="7" width="10.6328125" customWidth="1"/>
     <col min="10" max="10" width="12.6328125" customWidth="1"/>
     <col min="17" max="17" width="14.90625" customWidth="1"/>
-    <col min="18" max="18" width="8.1796875" customWidth="1"/>
+    <col min="18" max="18" width="78.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.35">

</xml_diff>